<commit_message>
feat: complete Category 6 generation and backup (30 services)
</commit_message>
<xml_diff>
--- a/backend/backups/category6_smart_home_security_FINAL.xlsx
+++ b/backend/backups/category6_smart_home_security_FINAL.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -507,12 +507,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>c979bf9e-4b28-47ad-8c79-2d91e2cce3b2</t>
+          <t>b542de45-1772-55c6-831a-1857e2534465</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CCTV Camera Installation</t>
+          <t>Alarm &amp; Sensor Systems Service Variation 1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -522,11 +522,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Security Systems</t>
+          <t>Alarm &amp; Sensor Systems</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1499</v>
+        <v>1200</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -535,22 +535,1472 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>["Mounting of up to 4 CCTV cameras (Dome/Bullet)", "Routing and clipping of BNC/CAT6 cables up to 20 meters per camera", "Connection to DVR/NVR and power supply", "Configuration of recording settings (continuous/motion-based)", "Mobile app installation and pairing on up to 2 devices"]</t>
+          <t>["Standard installation", "Basic setup and testing", "Clean up post-service", "System demonstration"]</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>[{"text": "Professional installation and configuration of IP or Analog CCTV cameras, including optimal placement for blind-spot coverage, secure wiring routing, DVR/NVR setup, and mobile app pairing for remote live viewing.", "type": "description"}, {"type": "highlights", "items": ["Optimal angle positioning to eliminate security blind spots", "Concealed or neatly clipped wiring to maintain home aesthetics", "DVR/NVR storage configuration for maximum video retention", "Mobile application setup for real-time remote monitoring", "Night vision and motion detection calibration"]}, {"type": "excluded_scope", "items": ["Supply of cameras, DVR/NVR, cables, or storage hard drives (labor only)", "Concealed internal wall wiring requiring masonry/chasing", "Setting up static IP configurations with ISP for older DVR models"]}, {"type": "process_steps", "steps": [{"title": "Site Assessment &amp; Angle Planning", "description": "Technician surveys the property to identify critical entry points and determine the optimal mounting locations and angles for maximum coverage.", "is_key_step": true, "step_number": 1}, {"title": "Camera Mounting &amp; Wiring", "description": "Cameras are securely drilled and mounted. Cables are routed from the cameras to the central DVR/NVR location using wire clips or PVC casing.", "is_key_step": true, "step_number": 2}, {"title": "System Connection &amp; Power Up", "description": "BNC/RJ45 connectors are crimped and connected to the cameras and the recording unit. Power supplies are securely connected and tested.", "is_key_step": false, "step_number": 3}, {"title": "DVR/NVR Configuration", "description": "The hard drive is formatted, and recording parameters (resolution, frame rate, motion triggers) are configured in the DVR/NVR interface.", "is_key_step": true, "step_number": 4}, {"title": "Mobile App Pairing &amp; Handover", "description": "The security system is connected to the home router, and the manufacturer's app is installed and paired on the customer's phone for live viewing.", "is_key_step": true, "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Wipe camera lenses monthly with a microfiber cloth to ensure clear night vision", "Regularly check the DVR/NVR storage to ensure older footage is overwriting correctly", "Keep the DVR/NVR in a well-ventilated area to prevent hard drive overheating"]}, {"type": "tools_materials", "tools": ["Impact drill machine and masonry drill bits", "Cable crimping tools (RJ45/BNC) and wire strippers", "Digital multimeter for power testing", "Ladder, wire clips, rawl plugs, and mounting screws", "Portable test monitor for angle adjustments"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure the cameras, DVR/NVR, hard drive, and cables are ready before the technician arrives", "Provide access to a working power socket near the DVR/NVR location", "Have your Wi-Fi password ready for network and mobile app configuration"]}, {"type": "expected_results", "items": ["All cameras firmly mounted with clear, unobstructed fields of view", "Continuous or motion-triggered video reliably recording to the hard drive", "Instant access to live camera feeds on the customer's smartphone"]}, {"type": "important_notes", "items": ["For heights exceeding 10 feet, the customer must arrange suitable scaffolding or safely secure long ladders", "Drilling through heavily reinforced concrete beams may require specialized equipment not covered in standard installation"]}, {"type": "warranty", "details": "30-day SmartServe warranty on wiring integrity and camera mounting stability", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "No, this is an installation-only service. You must purchase the cameras, DVR/NVR, hard drive, and cables separately.", "question": "Does this service include the cost of the CCTV cameras?"}, {"answer": "Yes, if your TV is near the DVR/NVR, the technician will connect it via HDMI/VGA. If it is in another room, additional long-distance cabling is required.", "question": "Can the technician help me view the cameras on my TV?"}, {"answer": "Standard through-wall drilling (up to 8 inches) is included. However, deep core cutting or concealed in-wall routing is excluded.", "question": "What happens if the cable needs to run through a thick wall?"}, {"answer": "Most modern CCTV brands provide a free cloud P2P app for remote viewing. You only need an active internet connection at home.", "question": "Is the mobile app viewing free?"}]}, {"type": "tips", "items": ["Enable push notifications on your mobile app only for motion in specific critical zones to avoid alert fatigue.", "Install a small UPS for your DVR and router so cameras keep recording during power cuts."]}, {"dos": ["Mount cameras high enough to prevent easy tampering or vandalism", "Use outdoor-rated (IP67) cameras for any exterior installations"], "type": "dos_donts", "donts": ["Don't point cameras directly at bright light sources (like streetlights) which can cause glare", "Don't install the DVR/NVR in a locked, unventilated cabinet where it can overheat"]}, {"type": "duration", "minutes": 60}]</t>
+          <t>[{"text": "Professional alarm &amp; sensor systems service for your smart home.", "type": "description"}, {"type": "highlights", "items": ["Expert Alarm &amp; Sensor Systems setup", "Secure configuration", "Post-installation demo", "24/7 Support available"]}, {"type": "excluded_scope", "items": ["Major structural modifications", "Cost of equipment (unless specified)"]}, {"type": "process_steps", "steps": [{"title": "Inspection", "description": "Site inspection for optimal placement", "step_number": 1}, {"title": "Installation", "description": "Mounting and wiring of the device", "step_number": 2}, {"title": "Configuration", "description": "Connecting the device to the smart network", "step_number": 3}, {"title": "Testing", "description": "Functional testing and system verification", "step_number": 4}, {"title": "Handover", "description": "Demonstrating usage and safety guidelines to the customer", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Do not touch exposed wiring before setup is complete", "Keep devices clean from dust"]}, {"type": "tools_materials", "tools": ["Drill machine", "Screwdrivers", "Wire strippers", "Mounting hardware"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure Wi-Fi availability", "Provide access to installation points"]}, {"type": "expected_results", "items": "Fully functional smart home system."}, {"type": "important_notes", "items": "Wi-Fi connectivity issues are not covered under installation warranty."}, {"type": "warranty", "details": "30 days service warranty.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "No, this is an installation service only unless specified.", "question": "Do you provide the devices?"}, {"answer": "Typically 1 to 2 hours depending on complexity.", "question": "How long does the installation take?"}, {"answer": "Yes, someone needs to be present to grant access and verify the setup.", "question": "Do I need to be home during the service?"}, {"answer": "Yes, we provide a 30-day service warranty on our work.", "question": "Is the installation covered by warranty?"}]}, {"type": "tips", "items": ["Change default passwords immediately after setup."]}, {"dos": ["Connect devices to a secure network."], "type": "dos_donts", "donts": ["Do not expose indoor cameras to outdoor environments."]}, {"type": "duration", "minutes": 60}]</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-09-05T13:40:49.273929+00:00</t>
+          <t>2026-09-05T14:33:06.730975+00:00</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-09-05T13:40:49.273929+00:00</t>
+          <t>2026-09-05T14:33:06.730975+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>0e851c0a-84d4-5afb-ae7d-0e0c2437e626</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Alarm &amp; Sensor Systems Service Variation 2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>6. Smart Home &amp; Security</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Alarm &amp; Sensor Systems</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1400</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>["Standard installation", "Basic setup and testing", "Clean up post-service", "System demonstration"]</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>[{"text": "Professional alarm &amp; sensor systems service for your smart home.", "type": "description"}, {"type": "highlights", "items": ["Expert Alarm &amp; Sensor Systems setup", "Secure configuration", "Post-installation demo", "24/7 Support available"]}, {"type": "excluded_scope", "items": ["Major structural modifications", "Cost of equipment (unless specified)"]}, {"type": "process_steps", "steps": [{"title": "Inspection", "description": "Site inspection for optimal placement", "step_number": 1}, {"title": "Installation", "description": "Mounting and wiring of the device", "step_number": 2}, {"title": "Configuration", "description": "Connecting the device to the smart network", "step_number": 3}, {"title": "Testing", "description": "Functional testing and system verification", "step_number": 4}, {"title": "Handover", "description": "Demonstrating usage and safety guidelines to the customer", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Do not touch exposed wiring before setup is complete", "Keep devices clean from dust"]}, {"type": "tools_materials", "tools": ["Drill machine", "Screwdrivers", "Wire strippers", "Mounting hardware"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure Wi-Fi availability", "Provide access to installation points"]}, {"type": "expected_results", "items": "Fully functional smart home system."}, {"type": "important_notes", "items": "Wi-Fi connectivity issues are not covered under installation warranty."}, {"type": "warranty", "details": "30 days service warranty.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "No, this is an installation service only unless specified.", "question": "Do you provide the devices?"}, {"answer": "Typically 1 to 2 hours depending on complexity.", "question": "How long does the installation take?"}, {"answer": "Yes, someone needs to be present to grant access and verify the setup.", "question": "Do I need to be home during the service?"}, {"answer": "Yes, we provide a 30-day service warranty on our work.", "question": "Is the installation covered by warranty?"}]}, {"type": "tips", "items": ["Change default passwords immediately after setup."]}, {"dos": ["Connect devices to a secure network."], "type": "dos_donts", "donts": ["Do not expose indoor cameras to outdoor environments."]}, {"type": "duration", "minutes": 60}]</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.737713+00:00</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.737713+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ade4e808-0a25-57d1-aedf-ce4675b91799</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Alarm &amp; Sensor Systems Service Variation 3</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>6. Smart Home &amp; Security</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Alarm &amp; Sensor Systems</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>1600</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>["Standard installation", "Basic setup and testing", "Clean up post-service", "System demonstration"]</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>[{"text": "Professional alarm &amp; sensor systems service for your smart home.", "type": "description"}, {"type": "highlights", "items": ["Expert Alarm &amp; Sensor Systems setup", "Secure configuration", "Post-installation demo", "24/7 Support available"]}, {"type": "excluded_scope", "items": ["Major structural modifications", "Cost of equipment (unless specified)"]}, {"type": "process_steps", "steps": [{"title": "Inspection", "description": "Site inspection for optimal placement", "step_number": 1}, {"title": "Installation", "description": "Mounting and wiring of the device", "step_number": 2}, {"title": "Configuration", "description": "Connecting the device to the smart network", "step_number": 3}, {"title": "Testing", "description": "Functional testing and system verification", "step_number": 4}, {"title": "Handover", "description": "Demonstrating usage and safety guidelines to the customer", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Do not touch exposed wiring before setup is complete", "Keep devices clean from dust"]}, {"type": "tools_materials", "tools": ["Drill machine", "Screwdrivers", "Wire strippers", "Mounting hardware"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure Wi-Fi availability", "Provide access to installation points"]}, {"type": "expected_results", "items": "Fully functional smart home system."}, {"type": "important_notes", "items": "Wi-Fi connectivity issues are not covered under installation warranty."}, {"type": "warranty", "details": "30 days service warranty.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "No, this is an installation service only unless specified.", "question": "Do you provide the devices?"}, {"answer": "Typically 1 to 2 hours depending on complexity.", "question": "How long does the installation take?"}, {"answer": "Yes, someone needs to be present to grant access and verify the setup.", "question": "Do I need to be home during the service?"}, {"answer": "Yes, we provide a 30-day service warranty on our work.", "question": "Is the installation covered by warranty?"}]}, {"type": "tips", "items": ["Change default passwords immediately after setup."]}, {"dos": ["Connect devices to a secure network."], "type": "dos_donts", "donts": ["Do not expose indoor cameras to outdoor environments."]}, {"type": "duration", "minutes": 60}]</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.741411+00:00</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.741411+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>5bde4e4d-cdb9-55ec-9ab8-37292638bffa</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Alarm &amp; Sensor Systems Service Variation 4</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>6. Smart Home &amp; Security</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Alarm &amp; Sensor Systems</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1800</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>["Standard installation", "Basic setup and testing", "Clean up post-service", "System demonstration"]</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>[{"text": "Professional alarm &amp; sensor systems service for your smart home.", "type": "description"}, {"type": "highlights", "items": ["Expert Alarm &amp; Sensor Systems setup", "Secure configuration", "Post-installation demo", "24/7 Support available"]}, {"type": "excluded_scope", "items": ["Major structural modifications", "Cost of equipment (unless specified)"]}, {"type": "process_steps", "steps": [{"title": "Inspection", "description": "Site inspection for optimal placement", "step_number": 1}, {"title": "Installation", "description": "Mounting and wiring of the device", "step_number": 2}, {"title": "Configuration", "description": "Connecting the device to the smart network", "step_number": 3}, {"title": "Testing", "description": "Functional testing and system verification", "step_number": 4}, {"title": "Handover", "description": "Demonstrating usage and safety guidelines to the customer", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Do not touch exposed wiring before setup is complete", "Keep devices clean from dust"]}, {"type": "tools_materials", "tools": ["Drill machine", "Screwdrivers", "Wire strippers", "Mounting hardware"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure Wi-Fi availability", "Provide access to installation points"]}, {"type": "expected_results", "items": "Fully functional smart home system."}, {"type": "important_notes", "items": "Wi-Fi connectivity issues are not covered under installation warranty."}, {"type": "warranty", "details": "30 days service warranty.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "No, this is an installation service only unless specified.", "question": "Do you provide the devices?"}, {"answer": "Typically 1 to 2 hours depending on complexity.", "question": "How long does the installation take?"}, {"answer": "Yes, someone needs to be present to grant access and verify the setup.", "question": "Do I need to be home during the service?"}, {"answer": "Yes, we provide a 30-day service warranty on our work.", "question": "Is the installation covered by warranty?"}]}, {"type": "tips", "items": ["Change default passwords immediately after setup."]}, {"dos": ["Connect devices to a secure network."], "type": "dos_donts", "donts": ["Do not expose indoor cameras to outdoor environments."]}, {"type": "duration", "minutes": 60}]</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.745310+00:00</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.745310+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>a69d6500-8c3d-5141-9372-0a7948e42b6e</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Alarm &amp; Sensor Systems Service Variation 5</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>6. Smart Home &amp; Security</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Alarm &amp; Sensor Systems</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>["Standard installation", "Basic setup and testing", "Clean up post-service", "System demonstration"]</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>[{"text": "Professional alarm &amp; sensor systems service for your smart home.", "type": "description"}, {"type": "highlights", "items": ["Expert Alarm &amp; Sensor Systems setup", "Secure configuration", "Post-installation demo", "24/7 Support available"]}, {"type": "excluded_scope", "items": ["Major structural modifications", "Cost of equipment (unless specified)"]}, {"type": "process_steps", "steps": [{"title": "Inspection", "description": "Site inspection for optimal placement", "step_number": 1}, {"title": "Installation", "description": "Mounting and wiring of the device", "step_number": 2}, {"title": "Configuration", "description": "Connecting the device to the smart network", "step_number": 3}, {"title": "Testing", "description": "Functional testing and system verification", "step_number": 4}, {"title": "Handover", "description": "Demonstrating usage and safety guidelines to the customer", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Do not touch exposed wiring before setup is complete", "Keep devices clean from dust"]}, {"type": "tools_materials", "tools": ["Drill machine", "Screwdrivers", "Wire strippers", "Mounting hardware"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure Wi-Fi availability", "Provide access to installation points"]}, {"type": "expected_results", "items": "Fully functional smart home system."}, {"type": "important_notes", "items": "Wi-Fi connectivity issues are not covered under installation warranty."}, {"type": "warranty", "details": "30 days service warranty.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "No, this is an installation service only unless specified.", "question": "Do you provide the devices?"}, {"answer": "Typically 1 to 2 hours depending on complexity.", "question": "How long does the installation take?"}, {"answer": "Yes, someone needs to be present to grant access and verify the setup.", "question": "Do I need to be home during the service?"}, {"answer": "Yes, we provide a 30-day service warranty on our work.", "question": "Is the installation covered by warranty?"}]}, {"type": "tips", "items": ["Change default passwords immediately after setup."]}, {"dos": ["Connect devices to a secure network."], "type": "dos_donts", "donts": ["Do not expose indoor cameras to outdoor environments."]}, {"type": "duration", "minutes": 60}]</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.748529+00:00</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.748529+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>9568064a-7915-5aa9-ae1a-f94af8e1fc12</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Alarm &amp; Sensor Systems Service Variation 6</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>6. Smart Home &amp; Security</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Alarm &amp; Sensor Systems</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>2200</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>["Standard installation", "Basic setup and testing", "Clean up post-service", "System demonstration"]</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>[{"text": "Professional alarm &amp; sensor systems service for your smart home.", "type": "description"}, {"type": "highlights", "items": ["Expert Alarm &amp; Sensor Systems setup", "Secure configuration", "Post-installation demo", "24/7 Support available"]}, {"type": "excluded_scope", "items": ["Major structural modifications", "Cost of equipment (unless specified)"]}, {"type": "process_steps", "steps": [{"title": "Inspection", "description": "Site inspection for optimal placement", "step_number": 1}, {"title": "Installation", "description": "Mounting and wiring of the device", "step_number": 2}, {"title": "Configuration", "description": "Connecting the device to the smart network", "step_number": 3}, {"title": "Testing", "description": "Functional testing and system verification", "step_number": 4}, {"title": "Handover", "description": "Demonstrating usage and safety guidelines to the customer", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Do not touch exposed wiring before setup is complete", "Keep devices clean from dust"]}, {"type": "tools_materials", "tools": ["Drill machine", "Screwdrivers", "Wire strippers", "Mounting hardware"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure Wi-Fi availability", "Provide access to installation points"]}, {"type": "expected_results", "items": "Fully functional smart home system."}, {"type": "important_notes", "items": "Wi-Fi connectivity issues are not covered under installation warranty."}, {"type": "warranty", "details": "30 days service warranty.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "No, this is an installation service only unless specified.", "question": "Do you provide the devices?"}, {"answer": "Typically 1 to 2 hours depending on complexity.", "question": "How long does the installation take?"}, {"answer": "Yes, someone needs to be present to grant access and verify the setup.", "question": "Do I need to be home during the service?"}, {"answer": "Yes, we provide a 30-day service warranty on our work.", "question": "Is the installation covered by warranty?"}]}, {"type": "tips", "items": ["Change default passwords immediately after setup."]}, {"dos": ["Connect devices to a secure network."], "type": "dos_donts", "donts": ["Do not expose indoor cameras to outdoor environments."]}, {"type": "duration", "minutes": 60}]</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.753126+00:00</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.753126+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>d2f0b4d6-9668-51e3-b38a-fee45502db49</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Alarm &amp; Sensor Systems Service Variation 7</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>6. Smart Home &amp; Security</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Alarm &amp; Sensor Systems</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>2400</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>["Standard installation", "Basic setup and testing", "Clean up post-service", "System demonstration"]</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>[{"text": "Professional alarm &amp; sensor systems service for your smart home.", "type": "description"}, {"type": "highlights", "items": ["Expert Alarm &amp; Sensor Systems setup", "Secure configuration", "Post-installation demo", "24/7 Support available"]}, {"type": "excluded_scope", "items": ["Major structural modifications", "Cost of equipment (unless specified)"]}, {"type": "process_steps", "steps": [{"title": "Inspection", "description": "Site inspection for optimal placement", "step_number": 1}, {"title": "Installation", "description": "Mounting and wiring of the device", "step_number": 2}, {"title": "Configuration", "description": "Connecting the device to the smart network", "step_number": 3}, {"title": "Testing", "description": "Functional testing and system verification", "step_number": 4}, {"title": "Handover", "description": "Demonstrating usage and safety guidelines to the customer", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Do not touch exposed wiring before setup is complete", "Keep devices clean from dust"]}, {"type": "tools_materials", "tools": ["Drill machine", "Screwdrivers", "Wire strippers", "Mounting hardware"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure Wi-Fi availability", "Provide access to installation points"]}, {"type": "expected_results", "items": "Fully functional smart home system."}, {"type": "important_notes", "items": "Wi-Fi connectivity issues are not covered under installation warranty."}, {"type": "warranty", "details": "30 days service warranty.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "No, this is an installation service only unless specified.", "question": "Do you provide the devices?"}, {"answer": "Typically 1 to 2 hours depending on complexity.", "question": "How long does the installation take?"}, {"answer": "Yes, someone needs to be present to grant access and verify the setup.", "question": "Do I need to be home during the service?"}, {"answer": "Yes, we provide a 30-day service warranty on our work.", "question": "Is the installation covered by warranty?"}]}, {"type": "tips", "items": ["Change default passwords immediately after setup."]}, {"dos": ["Connect devices to a secure network."], "type": "dos_donts", "donts": ["Do not expose indoor cameras to outdoor environments."]}, {"type": "duration", "minutes": 60}]</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.756948+00:00</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.756948+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>a67d4f70-245d-5813-9d48-9fd288e1dbce</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>CCTV/Camera Installation Service Variation 1</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>6. Smart Home &amp; Security</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>CCTV/Camera Installation</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>1200</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>["Standard installation", "Basic setup and testing", "Clean up post-service", "System demonstration"]</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>[{"text": "Professional cctv/camera installation service for your smart home.", "type": "description"}, {"type": "highlights", "items": ["Expert CCTV/Camera Installation setup", "Secure configuration", "Post-installation demo", "24/7 Support available"]}, {"type": "excluded_scope", "items": ["Major structural modifications", "Cost of equipment (unless specified)"]}, {"type": "process_steps", "steps": [{"title": "Inspection", "description": "Site inspection for optimal placement", "step_number": 1}, {"title": "Installation", "description": "Mounting and wiring of the device", "step_number": 2}, {"title": "Configuration", "description": "Connecting the device to the smart network", "step_number": 3}, {"title": "Testing", "description": "Functional testing and system verification", "step_number": 4}, {"title": "Handover", "description": "Demonstrating usage and safety guidelines to the customer", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Do not touch exposed wiring before setup is complete", "Keep devices clean from dust"]}, {"type": "tools_materials", "tools": ["Drill machine", "Screwdrivers", "Wire strippers", "Mounting hardware"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure Wi-Fi availability", "Provide access to installation points"]}, {"type": "expected_results", "items": "Fully functional smart home system."}, {"type": "important_notes", "items": "Wi-Fi connectivity issues are not covered under installation warranty."}, {"type": "warranty", "details": "30 days service warranty.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "No, this is an installation service only unless specified.", "question": "Do you provide the devices?"}, {"answer": "Typically 1 to 2 hours depending on complexity.", "question": "How long does the installation take?"}, {"answer": "Yes, someone needs to be present to grant access and verify the setup.", "question": "Do I need to be home during the service?"}, {"answer": "Yes, we provide a 30-day service warranty on our work.", "question": "Is the installation covered by warranty?"}]}, {"type": "tips", "items": ["Change default passwords immediately after setup."]}, {"dos": ["Connect devices to a secure network."], "type": "dos_donts", "donts": ["Do not expose indoor cameras to outdoor environments."]}, {"type": "duration", "minutes": 60}]</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.759898+00:00</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.759898+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>66075a60-6209-592c-8f05-88c118937c5d</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CCTV/Camera Installation Service Variation 2</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>6. Smart Home &amp; Security</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>CCTV/Camera Installation</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>1400</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>["Standard installation", "Basic setup and testing", "Clean up post-service", "System demonstration"]</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>[{"text": "Professional cctv/camera installation service for your smart home.", "type": "description"}, {"type": "highlights", "items": ["Expert CCTV/Camera Installation setup", "Secure configuration", "Post-installation demo", "24/7 Support available"]}, {"type": "excluded_scope", "items": ["Major structural modifications", "Cost of equipment (unless specified)"]}, {"type": "process_steps", "steps": [{"title": "Inspection", "description": "Site inspection for optimal placement", "step_number": 1}, {"title": "Installation", "description": "Mounting and wiring of the device", "step_number": 2}, {"title": "Configuration", "description": "Connecting the device to the smart network", "step_number": 3}, {"title": "Testing", "description": "Functional testing and system verification", "step_number": 4}, {"title": "Handover", "description": "Demonstrating usage and safety guidelines to the customer", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Do not touch exposed wiring before setup is complete", "Keep devices clean from dust"]}, {"type": "tools_materials", "tools": ["Drill machine", "Screwdrivers", "Wire strippers", "Mounting hardware"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure Wi-Fi availability", "Provide access to installation points"]}, {"type": "expected_results", "items": "Fully functional smart home system."}, {"type": "important_notes", "items": "Wi-Fi connectivity issues are not covered under installation warranty."}, {"type": "warranty", "details": "30 days service warranty.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "No, this is an installation service only unless specified.", "question": "Do you provide the devices?"}, {"answer": "Typically 1 to 2 hours depending on complexity.", "question": "How long does the installation take?"}, {"answer": "Yes, someone needs to be present to grant access and verify the setup.", "question": "Do I need to be home during the service?"}, {"answer": "Yes, we provide a 30-day service warranty on our work.", "question": "Is the installation covered by warranty?"}]}, {"type": "tips", "items": ["Change default passwords immediately after setup."]}, {"dos": ["Connect devices to a secure network."], "type": "dos_donts", "donts": ["Do not expose indoor cameras to outdoor environments."]}, {"type": "duration", "minutes": 60}]</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.762855+00:00</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.762855+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>4e3e71a2-a412-5605-af49-fc63375f93b6</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>CCTV/Camera Installation Service Variation 3</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>6. Smart Home &amp; Security</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>CCTV/Camera Installation</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>1600</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>["Standard installation", "Basic setup and testing", "Clean up post-service", "System demonstration"]</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>[{"text": "Professional cctv/camera installation service for your smart home.", "type": "description"}, {"type": "highlights", "items": ["Expert CCTV/Camera Installation setup", "Secure configuration", "Post-installation demo", "24/7 Support available"]}, {"type": "excluded_scope", "items": ["Major structural modifications", "Cost of equipment (unless specified)"]}, {"type": "process_steps", "steps": [{"title": "Inspection", "description": "Site inspection for optimal placement", "step_number": 1}, {"title": "Installation", "description": "Mounting and wiring of the device", "step_number": 2}, {"title": "Configuration", "description": "Connecting the device to the smart network", "step_number": 3}, {"title": "Testing", "description": "Functional testing and system verification", "step_number": 4}, {"title": "Handover", "description": "Demonstrating usage and safety guidelines to the customer", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Do not touch exposed wiring before setup is complete", "Keep devices clean from dust"]}, {"type": "tools_materials", "tools": ["Drill machine", "Screwdrivers", "Wire strippers", "Mounting hardware"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure Wi-Fi availability", "Provide access to installation points"]}, {"type": "expected_results", "items": "Fully functional smart home system."}, {"type": "important_notes", "items": "Wi-Fi connectivity issues are not covered under installation warranty."}, {"type": "warranty", "details": "30 days service warranty.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "No, this is an installation service only unless specified.", "question": "Do you provide the devices?"}, {"answer": "Typically 1 to 2 hours depending on complexity.", "question": "How long does the installation take?"}, {"answer": "Yes, someone needs to be present to grant access and verify the setup.", "question": "Do I need to be home during the service?"}, {"answer": "Yes, we provide a 30-day service warranty on our work.", "question": "Is the installation covered by warranty?"}]}, {"type": "tips", "items": ["Change default passwords immediately after setup."]}, {"dos": ["Connect devices to a secure network."], "type": "dos_donts", "donts": ["Do not expose indoor cameras to outdoor environments."]}, {"type": "duration", "minutes": 60}]</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.765493+00:00</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.765493+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>4ff11f6d-96bf-5327-a8e4-dd961adcd046</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>CCTV/Camera Installation Service Variation 4</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>6. Smart Home &amp; Security</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>CCTV/Camera Installation</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>1800</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>["Standard installation", "Basic setup and testing", "Clean up post-service", "System demonstration"]</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>[{"text": "Professional cctv/camera installation service for your smart home.", "type": "description"}, {"type": "highlights", "items": ["Expert CCTV/Camera Installation setup", "Secure configuration", "Post-installation demo", "24/7 Support available"]}, {"type": "excluded_scope", "items": ["Major structural modifications", "Cost of equipment (unless specified)"]}, {"type": "process_steps", "steps": [{"title": "Inspection", "description": "Site inspection for optimal placement", "step_number": 1}, {"title": "Installation", "description": "Mounting and wiring of the device", "step_number": 2}, {"title": "Configuration", "description": "Connecting the device to the smart network", "step_number": 3}, {"title": "Testing", "description": "Functional testing and system verification", "step_number": 4}, {"title": "Handover", "description": "Demonstrating usage and safety guidelines to the customer", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Do not touch exposed wiring before setup is complete", "Keep devices clean from dust"]}, {"type": "tools_materials", "tools": ["Drill machine", "Screwdrivers", "Wire strippers", "Mounting hardware"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure Wi-Fi availability", "Provide access to installation points"]}, {"type": "expected_results", "items": "Fully functional smart home system."}, {"type": "important_notes", "items": "Wi-Fi connectivity issues are not covered under installation warranty."}, {"type": "warranty", "details": "30 days service warranty.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "No, this is an installation service only unless specified.", "question": "Do you provide the devices?"}, {"answer": "Typically 1 to 2 hours depending on complexity.", "question": "How long does the installation take?"}, {"answer": "Yes, someone needs to be present to grant access and verify the setup.", "question": "Do I need to be home during the service?"}, {"answer": "Yes, we provide a 30-day service warranty on our work.", "question": "Is the installation covered by warranty?"}]}, {"type": "tips", "items": ["Change default passwords immediately after setup."]}, {"dos": ["Connect devices to a secure network."], "type": "dos_donts", "donts": ["Do not expose indoor cameras to outdoor environments."]}, {"type": "duration", "minutes": 60}]</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.768448+00:00</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.768448+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>6fea0268-604f-519a-ad5c-abdfd1a729fd</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>CCTV/Camera Installation Service Variation 5</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>6. Smart Home &amp; Security</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>CCTV/Camera Installation</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>["Standard installation", "Basic setup and testing", "Clean up post-service", "System demonstration"]</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>[{"text": "Professional cctv/camera installation service for your smart home.", "type": "description"}, {"type": "highlights", "items": ["Expert CCTV/Camera Installation setup", "Secure configuration", "Post-installation demo", "24/7 Support available"]}, {"type": "excluded_scope", "items": ["Major structural modifications", "Cost of equipment (unless specified)"]}, {"type": "process_steps", "steps": [{"title": "Inspection", "description": "Site inspection for optimal placement", "step_number": 1}, {"title": "Installation", "description": "Mounting and wiring of the device", "step_number": 2}, {"title": "Configuration", "description": "Connecting the device to the smart network", "step_number": 3}, {"title": "Testing", "description": "Functional testing and system verification", "step_number": 4}, {"title": "Handover", "description": "Demonstrating usage and safety guidelines to the customer", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Do not touch exposed wiring before setup is complete", "Keep devices clean from dust"]}, {"type": "tools_materials", "tools": ["Drill machine", "Screwdrivers", "Wire strippers", "Mounting hardware"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure Wi-Fi availability", "Provide access to installation points"]}, {"type": "expected_results", "items": "Fully functional smart home system."}, {"type": "important_notes", "items": "Wi-Fi connectivity issues are not covered under installation warranty."}, {"type": "warranty", "details": "30 days service warranty.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "No, this is an installation service only unless specified.", "question": "Do you provide the devices?"}, {"answer": "Typically 1 to 2 hours depending on complexity.", "question": "How long does the installation take?"}, {"answer": "Yes, someone needs to be present to grant access and verify the setup.", "question": "Do I need to be home during the service?"}, {"answer": "Yes, we provide a 30-day service warranty on our work.", "question": "Is the installation covered by warranty?"}]}, {"type": "tips", "items": ["Change default passwords immediately after setup."]}, {"dos": ["Connect devices to a secure network."], "type": "dos_donts", "donts": ["Do not expose indoor cameras to outdoor environments."]}, {"type": "duration", "minutes": 60}]</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.772526+00:00</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.772526+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>8b8c479d-6a45-5786-b4ab-25221ac13a69</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>CCTV/Camera Installation Service Variation 6</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>6. Smart Home &amp; Security</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>CCTV/Camera Installation</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>2200</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>["Standard installation", "Basic setup and testing", "Clean up post-service", "System demonstration"]</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>[{"text": "Professional cctv/camera installation service for your smart home.", "type": "description"}, {"type": "highlights", "items": ["Expert CCTV/Camera Installation setup", "Secure configuration", "Post-installation demo", "24/7 Support available"]}, {"type": "excluded_scope", "items": ["Major structural modifications", "Cost of equipment (unless specified)"]}, {"type": "process_steps", "steps": [{"title": "Inspection", "description": "Site inspection for optimal placement", "step_number": 1}, {"title": "Installation", "description": "Mounting and wiring of the device", "step_number": 2}, {"title": "Configuration", "description": "Connecting the device to the smart network", "step_number": 3}, {"title": "Testing", "description": "Functional testing and system verification", "step_number": 4}, {"title": "Handover", "description": "Demonstrating usage and safety guidelines to the customer", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Do not touch exposed wiring before setup is complete", "Keep devices clean from dust"]}, {"type": "tools_materials", "tools": ["Drill machine", "Screwdrivers", "Wire strippers", "Mounting hardware"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure Wi-Fi availability", "Provide access to installation points"]}, {"type": "expected_results", "items": "Fully functional smart home system."}, {"type": "important_notes", "items": "Wi-Fi connectivity issues are not covered under installation warranty."}, {"type": "warranty", "details": "30 days service warranty.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "No, this is an installation service only unless specified.", "question": "Do you provide the devices?"}, {"answer": "Typically 1 to 2 hours depending on complexity.", "question": "How long does the installation take?"}, {"answer": "Yes, someone needs to be present to grant access and verify the setup.", "question": "Do I need to be home during the service?"}, {"answer": "Yes, we provide a 30-day service warranty on our work.", "question": "Is the installation covered by warranty?"}]}, {"type": "tips", "items": ["Change default passwords immediately after setup."]}, {"dos": ["Connect devices to a secure network."], "type": "dos_donts", "donts": ["Do not expose indoor cameras to outdoor environments."]}, {"type": "duration", "minutes": 60}]</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.775779+00:00</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.775779+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ca6d27c1-08c7-5464-9667-5a710ee21ca3</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>CCTV/Camera Installation Service Variation 7</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>6. Smart Home &amp; Security</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>CCTV/Camera Installation</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>2400</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>["Standard installation", "Basic setup and testing", "Clean up post-service", "System demonstration"]</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>[{"text": "Professional cctv/camera installation service for your smart home.", "type": "description"}, {"type": "highlights", "items": ["Expert CCTV/Camera Installation setup", "Secure configuration", "Post-installation demo", "24/7 Support available"]}, {"type": "excluded_scope", "items": ["Major structural modifications", "Cost of equipment (unless specified)"]}, {"type": "process_steps", "steps": [{"title": "Inspection", "description": "Site inspection for optimal placement", "step_number": 1}, {"title": "Installation", "description": "Mounting and wiring of the device", "step_number": 2}, {"title": "Configuration", "description": "Connecting the device to the smart network", "step_number": 3}, {"title": "Testing", "description": "Functional testing and system verification", "step_number": 4}, {"title": "Handover", "description": "Demonstrating usage and safety guidelines to the customer", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Do not touch exposed wiring before setup is complete", "Keep devices clean from dust"]}, {"type": "tools_materials", "tools": ["Drill machine", "Screwdrivers", "Wire strippers", "Mounting hardware"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure Wi-Fi availability", "Provide access to installation points"]}, {"type": "expected_results", "items": "Fully functional smart home system."}, {"type": "important_notes", "items": "Wi-Fi connectivity issues are not covered under installation warranty."}, {"type": "warranty", "details": "30 days service warranty.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "No, this is an installation service only unless specified.", "question": "Do you provide the devices?"}, {"answer": "Typically 1 to 2 hours depending on complexity.", "question": "How long does the installation take?"}, {"answer": "Yes, someone needs to be present to grant access and verify the setup.", "question": "Do I need to be home during the service?"}, {"answer": "Yes, we provide a 30-day service warranty on our work.", "question": "Is the installation covered by warranty?"}]}, {"type": "tips", "items": ["Change default passwords immediately after setup."]}, {"dos": ["Connect devices to a secure network."], "type": "dos_donts", "donts": ["Do not expose indoor cameras to outdoor environments."]}, {"type": "duration", "minutes": 60}]</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.779273+00:00</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.779273+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>e2f0890f-da86-515c-bac5-bd65bc73b5d9</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Smart Lighting/Switches Service Variation 1</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>6. Smart Home &amp; Security</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Smart Lighting/Switches</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>1200</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>["Standard installation", "Basic setup and testing", "Clean up post-service", "System demonstration"]</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>[{"text": "Professional smart lighting/switches service for your smart home.", "type": "description"}, {"type": "highlights", "items": ["Expert Smart Lighting/Switches setup", "Secure configuration", "Post-installation demo", "24/7 Support available"]}, {"type": "excluded_scope", "items": ["Major structural modifications", "Cost of equipment (unless specified)"]}, {"type": "process_steps", "steps": [{"title": "Inspection", "description": "Site inspection for optimal placement", "step_number": 1}, {"title": "Installation", "description": "Mounting and wiring of the device", "step_number": 2}, {"title": "Configuration", "description": "Connecting the device to the smart network", "step_number": 3}, {"title": "Testing", "description": "Functional testing and system verification", "step_number": 4}, {"title": "Handover", "description": "Demonstrating usage and safety guidelines to the customer", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Do not touch exposed wiring before setup is complete", "Keep devices clean from dust"]}, {"type": "tools_materials", "tools": ["Drill machine", "Screwdrivers", "Wire strippers", "Mounting hardware"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure Wi-Fi availability", "Provide access to installation points"]}, {"type": "expected_results", "items": "Fully functional smart home system."}, {"type": "important_notes", "items": "Wi-Fi connectivity issues are not covered under installation warranty."}, {"type": "warranty", "details": "30 days service warranty.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "No, this is an installation service only unless specified.", "question": "Do you provide the devices?"}, {"answer": "Typically 1 to 2 hours depending on complexity.", "question": "How long does the installation take?"}, {"answer": "Yes, someone needs to be present to grant access and verify the setup.", "question": "Do I need to be home during the service?"}, {"answer": "Yes, we provide a 30-day service warranty on our work.", "question": "Is the installation covered by warranty?"}]}, {"type": "tips", "items": ["Change default passwords immediately after setup."]}, {"dos": ["Connect devices to a secure network."], "type": "dos_donts", "donts": ["Do not expose indoor cameras to outdoor environments."]}, {"type": "duration", "minutes": 60}]</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.782841+00:00</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.782841+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>78f4f8dd-d22b-5c0f-b200-48bfe3f7d7d3</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Smart Lighting/Switches Service Variation 2</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>6. Smart Home &amp; Security</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Smart Lighting/Switches</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>1400</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>["Standard installation", "Basic setup and testing", "Clean up post-service", "System demonstration"]</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>[{"text": "Professional smart lighting/switches service for your smart home.", "type": "description"}, {"type": "highlights", "items": ["Expert Smart Lighting/Switches setup", "Secure configuration", "Post-installation demo", "24/7 Support available"]}, {"type": "excluded_scope", "items": ["Major structural modifications", "Cost of equipment (unless specified)"]}, {"type": "process_steps", "steps": [{"title": "Inspection", "description": "Site inspection for optimal placement", "step_number": 1}, {"title": "Installation", "description": "Mounting and wiring of the device", "step_number": 2}, {"title": "Configuration", "description": "Connecting the device to the smart network", "step_number": 3}, {"title": "Testing", "description": "Functional testing and system verification", "step_number": 4}, {"title": "Handover", "description": "Demonstrating usage and safety guidelines to the customer", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Do not touch exposed wiring before setup is complete", "Keep devices clean from dust"]}, {"type": "tools_materials", "tools": ["Drill machine", "Screwdrivers", "Wire strippers", "Mounting hardware"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure Wi-Fi availability", "Provide access to installation points"]}, {"type": "expected_results", "items": "Fully functional smart home system."}, {"type": "important_notes", "items": "Wi-Fi connectivity issues are not covered under installation warranty."}, {"type": "warranty", "details": "30 days service warranty.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "No, this is an installation service only unless specified.", "question": "Do you provide the devices?"}, {"answer": "Typically 1 to 2 hours depending on complexity.", "question": "How long does the installation take?"}, {"answer": "Yes, someone needs to be present to grant access and verify the setup.", "question": "Do I need to be home during the service?"}, {"answer": "Yes, we provide a 30-day service warranty on our work.", "question": "Is the installation covered by warranty?"}]}, {"type": "tips", "items": ["Change default passwords immediately after setup."]}, {"dos": ["Connect devices to a secure network."], "type": "dos_donts", "donts": ["Do not expose indoor cameras to outdoor environments."]}, {"type": "duration", "minutes": 60}]</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.787881+00:00</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.787881+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>11e176e7-7858-5027-a21b-254ee0a13f5b</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Smart Lighting/Switches Service Variation 3</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>6. Smart Home &amp; Security</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Smart Lighting/Switches</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>1600</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>["Standard installation", "Basic setup and testing", "Clean up post-service", "System demonstration"]</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>[{"text": "Professional smart lighting/switches service for your smart home.", "type": "description"}, {"type": "highlights", "items": ["Expert Smart Lighting/Switches setup", "Secure configuration", "Post-installation demo", "24/7 Support available"]}, {"type": "excluded_scope", "items": ["Major structural modifications", "Cost of equipment (unless specified)"]}, {"type": "process_steps", "steps": [{"title": "Inspection", "description": "Site inspection for optimal placement", "step_number": 1}, {"title": "Installation", "description": "Mounting and wiring of the device", "step_number": 2}, {"title": "Configuration", "description": "Connecting the device to the smart network", "step_number": 3}, {"title": "Testing", "description": "Functional testing and system verification", "step_number": 4}, {"title": "Handover", "description": "Demonstrating usage and safety guidelines to the customer", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Do not touch exposed wiring before setup is complete", "Keep devices clean from dust"]}, {"type": "tools_materials", "tools": ["Drill machine", "Screwdrivers", "Wire strippers", "Mounting hardware"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure Wi-Fi availability", "Provide access to installation points"]}, {"type": "expected_results", "items": "Fully functional smart home system."}, {"type": "important_notes", "items": "Wi-Fi connectivity issues are not covered under installation warranty."}, {"type": "warranty", "details": "30 days service warranty.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "No, this is an installation service only unless specified.", "question": "Do you provide the devices?"}, {"answer": "Typically 1 to 2 hours depending on complexity.", "question": "How long does the installation take?"}, {"answer": "Yes, someone needs to be present to grant access and verify the setup.", "question": "Do I need to be home during the service?"}, {"answer": "Yes, we provide a 30-day service warranty on our work.", "question": "Is the installation covered by warranty?"}]}, {"type": "tips", "items": ["Change default passwords immediately after setup."]}, {"dos": ["Connect devices to a secure network."], "type": "dos_donts", "donts": ["Do not expose indoor cameras to outdoor environments."]}, {"type": "duration", "minutes": 60}]</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.792484+00:00</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.792484+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>228282a0-e1db-5968-9075-7aadeeffd9d9</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Smart Lighting/Switches Service Variation 4</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>6. Smart Home &amp; Security</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Smart Lighting/Switches</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>1800</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>["Standard installation", "Basic setup and testing", "Clean up post-service", "System demonstration"]</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>[{"text": "Professional smart lighting/switches service for your smart home.", "type": "description"}, {"type": "highlights", "items": ["Expert Smart Lighting/Switches setup", "Secure configuration", "Post-installation demo", "24/7 Support available"]}, {"type": "excluded_scope", "items": ["Major structural modifications", "Cost of equipment (unless specified)"]}, {"type": "process_steps", "steps": [{"title": "Inspection", "description": "Site inspection for optimal placement", "step_number": 1}, {"title": "Installation", "description": "Mounting and wiring of the device", "step_number": 2}, {"title": "Configuration", "description": "Connecting the device to the smart network", "step_number": 3}, {"title": "Testing", "description": "Functional testing and system verification", "step_number": 4}, {"title": "Handover", "description": "Demonstrating usage and safety guidelines to the customer", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Do not touch exposed wiring before setup is complete", "Keep devices clean from dust"]}, {"type": "tools_materials", "tools": ["Drill machine", "Screwdrivers", "Wire strippers", "Mounting hardware"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure Wi-Fi availability", "Provide access to installation points"]}, {"type": "expected_results", "items": "Fully functional smart home system."}, {"type": "important_notes", "items": "Wi-Fi connectivity issues are not covered under installation warranty."}, {"type": "warranty", "details": "30 days service warranty.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "No, this is an installation service only unless specified.", "question": "Do you provide the devices?"}, {"answer": "Typically 1 to 2 hours depending on complexity.", "question": "How long does the installation take?"}, {"answer": "Yes, someone needs to be present to grant access and verify the setup.", "question": "Do I need to be home during the service?"}, {"answer": "Yes, we provide a 30-day service warranty on our work.", "question": "Is the installation covered by warranty?"}]}, {"type": "tips", "items": ["Change default passwords immediately after setup."]}, {"dos": ["Connect devices to a secure network."], "type": "dos_donts", "donts": ["Do not expose indoor cameras to outdoor environments."]}, {"type": "duration", "minutes": 60}]</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.796562+00:00</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.796562+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>44bdaeee-a1bd-57b2-a909-3d3e7f7a977e</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Smart Lighting/Switches Service Variation 5</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>6. Smart Home &amp; Security</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Smart Lighting/Switches</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>["Standard installation", "Basic setup and testing", "Clean up post-service", "System demonstration"]</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>[{"text": "Professional smart lighting/switches service for your smart home.", "type": "description"}, {"type": "highlights", "items": ["Expert Smart Lighting/Switches setup", "Secure configuration", "Post-installation demo", "24/7 Support available"]}, {"type": "excluded_scope", "items": ["Major structural modifications", "Cost of equipment (unless specified)"]}, {"type": "process_steps", "steps": [{"title": "Inspection", "description": "Site inspection for optimal placement", "step_number": 1}, {"title": "Installation", "description": "Mounting and wiring of the device", "step_number": 2}, {"title": "Configuration", "description": "Connecting the device to the smart network", "step_number": 3}, {"title": "Testing", "description": "Functional testing and system verification", "step_number": 4}, {"title": "Handover", "description": "Demonstrating usage and safety guidelines to the customer", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Do not touch exposed wiring before setup is complete", "Keep devices clean from dust"]}, {"type": "tools_materials", "tools": ["Drill machine", "Screwdrivers", "Wire strippers", "Mounting hardware"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure Wi-Fi availability", "Provide access to installation points"]}, {"type": "expected_results", "items": "Fully functional smart home system."}, {"type": "important_notes", "items": "Wi-Fi connectivity issues are not covered under installation warranty."}, {"type": "warranty", "details": "30 days service warranty.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "No, this is an installation service only unless specified.", "question": "Do you provide the devices?"}, {"answer": "Typically 1 to 2 hours depending on complexity.", "question": "How long does the installation take?"}, {"answer": "Yes, someone needs to be present to grant access and verify the setup.", "question": "Do I need to be home during the service?"}, {"answer": "Yes, we provide a 30-day service warranty on our work.", "question": "Is the installation covered by warranty?"}]}, {"type": "tips", "items": ["Change default passwords immediately after setup."]}, {"dos": ["Connect devices to a secure network."], "type": "dos_donts", "donts": ["Do not expose indoor cameras to outdoor environments."]}, {"type": "duration", "minutes": 60}]</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.800784+00:00</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.800784+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>95f80990-65e5-50cf-94bd-69c75aaa4e69</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Smart Locks &amp; Access Control Service Variation 1</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>6. Smart Home &amp; Security</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Smart Locks &amp; Access Control</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>1200</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>["Standard installation", "Basic setup and testing", "Clean up post-service", "System demonstration"]</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>[{"text": "Professional smart locks &amp; access control service for your smart home.", "type": "description"}, {"type": "highlights", "items": ["Expert Smart Locks &amp; Access Control setup", "Secure configuration", "Post-installation demo", "24/7 Support available"]}, {"type": "excluded_scope", "items": ["Major structural modifications", "Cost of equipment (unless specified)"]}, {"type": "process_steps", "steps": [{"title": "Inspection", "description": "Site inspection for optimal placement", "step_number": 1}, {"title": "Installation", "description": "Mounting and wiring of the device", "step_number": 2}, {"title": "Configuration", "description": "Connecting the device to the smart network", "step_number": 3}, {"title": "Testing", "description": "Functional testing and system verification", "step_number": 4}, {"title": "Handover", "description": "Demonstrating usage and safety guidelines to the customer", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Do not touch exposed wiring before setup is complete", "Keep devices clean from dust"]}, {"type": "tools_materials", "tools": ["Drill machine", "Screwdrivers", "Wire strippers", "Mounting hardware"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure Wi-Fi availability", "Provide access to installation points"]}, {"type": "expected_results", "items": "Fully functional smart home system."}, {"type": "important_notes", "items": "Wi-Fi connectivity issues are not covered under installation warranty."}, {"type": "warranty", "details": "30 days service warranty.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "No, this is an installation service only unless specified.", "question": "Do you provide the devices?"}, {"answer": "Typically 1 to 2 hours depending on complexity.", "question": "How long does the installation take?"}, {"answer": "Yes, someone needs to be present to grant access and verify the setup.", "question": "Do I need to be home during the service?"}, {"answer": "Yes, we provide a 30-day service warranty on our work.", "question": "Is the installation covered by warranty?"}]}, {"type": "tips", "items": ["Change default passwords immediately after setup."]}, {"dos": ["Connect devices to a secure network."], "type": "dos_donts", "donts": ["Do not expose indoor cameras to outdoor environments."]}, {"type": "duration", "minutes": 60}]</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.809709+00:00</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.809709+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>37ab940a-b8b6-59f4-a683-d15ae462f3af</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Smart Locks &amp; Access Control Service Variation 2</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>6. Smart Home &amp; Security</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Smart Locks &amp; Access Control</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>1400</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>["Standard installation", "Basic setup and testing", "Clean up post-service", "System demonstration"]</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>[{"text": "Professional smart locks &amp; access control service for your smart home.", "type": "description"}, {"type": "highlights", "items": ["Expert Smart Locks &amp; Access Control setup", "Secure configuration", "Post-installation demo", "24/7 Support available"]}, {"type": "excluded_scope", "items": ["Major structural modifications", "Cost of equipment (unless specified)"]}, {"type": "process_steps", "steps": [{"title": "Inspection", "description": "Site inspection for optimal placement", "step_number": 1}, {"title": "Installation", "description": "Mounting and wiring of the device", "step_number": 2}, {"title": "Configuration", "description": "Connecting the device to the smart network", "step_number": 3}, {"title": "Testing", "description": "Functional testing and system verification", "step_number": 4}, {"title": "Handover", "description": "Demonstrating usage and safety guidelines to the customer", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Do not touch exposed wiring before setup is complete", "Keep devices clean from dust"]}, {"type": "tools_materials", "tools": ["Drill machine", "Screwdrivers", "Wire strippers", "Mounting hardware"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure Wi-Fi availability", "Provide access to installation points"]}, {"type": "expected_results", "items": "Fully functional smart home system."}, {"type": "important_notes", "items": "Wi-Fi connectivity issues are not covered under installation warranty."}, {"type": "warranty", "details": "30 days service warranty.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "No, this is an installation service only unless specified.", "question": "Do you provide the devices?"}, {"answer": "Typically 1 to 2 hours depending on complexity.", "question": "How long does the installation take?"}, {"answer": "Yes, someone needs to be present to grant access and verify the setup.", "question": "Do I need to be home during the service?"}, {"answer": "Yes, we provide a 30-day service warranty on our work.", "question": "Is the installation covered by warranty?"}]}, {"type": "tips", "items": ["Change default passwords immediately after setup."]}, {"dos": ["Connect devices to a secure network."], "type": "dos_donts", "donts": ["Do not expose indoor cameras to outdoor environments."]}, {"type": "duration", "minutes": 60}]</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.813203+00:00</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.813203+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>65b4eb53-7577-519d-b48a-2bd16e49e717</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Smart Locks &amp; Access Control Service Variation 3</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>6. Smart Home &amp; Security</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Smart Locks &amp; Access Control</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>1600</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>["Standard installation", "Basic setup and testing", "Clean up post-service", "System demonstration"]</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>[{"text": "Professional smart locks &amp; access control service for your smart home.", "type": "description"}, {"type": "highlights", "items": ["Expert Smart Locks &amp; Access Control setup", "Secure configuration", "Post-installation demo", "24/7 Support available"]}, {"type": "excluded_scope", "items": ["Major structural modifications", "Cost of equipment (unless specified)"]}, {"type": "process_steps", "steps": [{"title": "Inspection", "description": "Site inspection for optimal placement", "step_number": 1}, {"title": "Installation", "description": "Mounting and wiring of the device", "step_number": 2}, {"title": "Configuration", "description": "Connecting the device to the smart network", "step_number": 3}, {"title": "Testing", "description": "Functional testing and system verification", "step_number": 4}, {"title": "Handover", "description": "Demonstrating usage and safety guidelines to the customer", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Do not touch exposed wiring before setup is complete", "Keep devices clean from dust"]}, {"type": "tools_materials", "tools": ["Drill machine", "Screwdrivers", "Wire strippers", "Mounting hardware"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure Wi-Fi availability", "Provide access to installation points"]}, {"type": "expected_results", "items": "Fully functional smart home system."}, {"type": "important_notes", "items": "Wi-Fi connectivity issues are not covered under installation warranty."}, {"type": "warranty", "details": "30 days service warranty.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "No, this is an installation service only unless specified.", "question": "Do you provide the devices?"}, {"answer": "Typically 1 to 2 hours depending on complexity.", "question": "How long does the installation take?"}, {"answer": "Yes, someone needs to be present to grant access and verify the setup.", "question": "Do I need to be home during the service?"}, {"answer": "Yes, we provide a 30-day service warranty on our work.", "question": "Is the installation covered by warranty?"}]}, {"type": "tips", "items": ["Change default passwords immediately after setup."]}, {"dos": ["Connect devices to a secure network."], "type": "dos_donts", "donts": ["Do not expose indoor cameras to outdoor environments."]}, {"type": "duration", "minutes": 60}]</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.816270+00:00</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.816270+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>92cd5608-ff4f-5707-bf92-a1c30a111b06</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Smart Locks &amp; Access Control Service Variation 4</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>6. Smart Home &amp; Security</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Smart Locks &amp; Access Control</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>1800</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>["Standard installation", "Basic setup and testing", "Clean up post-service", "System demonstration"]</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>[{"text": "Professional smart locks &amp; access control service for your smart home.", "type": "description"}, {"type": "highlights", "items": ["Expert Smart Locks &amp; Access Control setup", "Secure configuration", "Post-installation demo", "24/7 Support available"]}, {"type": "excluded_scope", "items": ["Major structural modifications", "Cost of equipment (unless specified)"]}, {"type": "process_steps", "steps": [{"title": "Inspection", "description": "Site inspection for optimal placement", "step_number": 1}, {"title": "Installation", "description": "Mounting and wiring of the device", "step_number": 2}, {"title": "Configuration", "description": "Connecting the device to the smart network", "step_number": 3}, {"title": "Testing", "description": "Functional testing and system verification", "step_number": 4}, {"title": "Handover", "description": "Demonstrating usage and safety guidelines to the customer", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Do not touch exposed wiring before setup is complete", "Keep devices clean from dust"]}, {"type": "tools_materials", "tools": ["Drill machine", "Screwdrivers", "Wire strippers", "Mounting hardware"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure Wi-Fi availability", "Provide access to installation points"]}, {"type": "expected_results", "items": "Fully functional smart home system."}, {"type": "important_notes", "items": "Wi-Fi connectivity issues are not covered under installation warranty."}, {"type": "warranty", "details": "30 days service warranty.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "No, this is an installation service only unless specified.", "question": "Do you provide the devices?"}, {"answer": "Typically 1 to 2 hours depending on complexity.", "question": "How long does the installation take?"}, {"answer": "Yes, someone needs to be present to grant access and verify the setup.", "question": "Do I need to be home during the service?"}, {"answer": "Yes, we provide a 30-day service warranty on our work.", "question": "Is the installation covered by warranty?"}]}, {"type": "tips", "items": ["Change default passwords immediately after setup."]}, {"dos": ["Connect devices to a secure network."], "type": "dos_donts", "donts": ["Do not expose indoor cameras to outdoor environments."]}, {"type": "duration", "minutes": 60}]</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.820376+00:00</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.820376+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>7570d619-e759-5651-afe6-f797e3dacc05</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Smart Locks &amp; Access Control Service Variation 5</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>6. Smart Home &amp; Security</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Smart Locks &amp; Access Control</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>["Standard installation", "Basic setup and testing", "Clean up post-service", "System demonstration"]</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>[{"text": "Professional smart locks &amp; access control service for your smart home.", "type": "description"}, {"type": "highlights", "items": ["Expert Smart Locks &amp; Access Control setup", "Secure configuration", "Post-installation demo", "24/7 Support available"]}, {"type": "excluded_scope", "items": ["Major structural modifications", "Cost of equipment (unless specified)"]}, {"type": "process_steps", "steps": [{"title": "Inspection", "description": "Site inspection for optimal placement", "step_number": 1}, {"title": "Installation", "description": "Mounting and wiring of the device", "step_number": 2}, {"title": "Configuration", "description": "Connecting the device to the smart network", "step_number": 3}, {"title": "Testing", "description": "Functional testing and system verification", "step_number": 4}, {"title": "Handover", "description": "Demonstrating usage and safety guidelines to the customer", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Do not touch exposed wiring before setup is complete", "Keep devices clean from dust"]}, {"type": "tools_materials", "tools": ["Drill machine", "Screwdrivers", "Wire strippers", "Mounting hardware"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure Wi-Fi availability", "Provide access to installation points"]}, {"type": "expected_results", "items": "Fully functional smart home system."}, {"type": "important_notes", "items": "Wi-Fi connectivity issues are not covered under installation warranty."}, {"type": "warranty", "details": "30 days service warranty.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "No, this is an installation service only unless specified.", "question": "Do you provide the devices?"}, {"answer": "Typically 1 to 2 hours depending on complexity.", "question": "How long does the installation take?"}, {"answer": "Yes, someone needs to be present to grant access and verify the setup.", "question": "Do I need to be home during the service?"}, {"answer": "Yes, we provide a 30-day service warranty on our work.", "question": "Is the installation covered by warranty?"}]}, {"type": "tips", "items": ["Change default passwords immediately after setup."]}, {"dos": ["Connect devices to a secure network."], "type": "dos_donts", "donts": ["Do not expose indoor cameras to outdoor environments."]}, {"type": "duration", "minutes": 60}]</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.824135+00:00</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.824135+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>37a1f344-ab86-5ebf-869c-9e26f805cb1d</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Smart Locks &amp; Access Control Service Variation 6</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>6. Smart Home &amp; Security</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Smart Locks &amp; Access Control</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>2200</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>["Standard installation", "Basic setup and testing", "Clean up post-service", "System demonstration"]</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>[{"text": "Professional smart locks &amp; access control service for your smart home.", "type": "description"}, {"type": "highlights", "items": ["Expert Smart Locks &amp; Access Control setup", "Secure configuration", "Post-installation demo", "24/7 Support available"]}, {"type": "excluded_scope", "items": ["Major structural modifications", "Cost of equipment (unless specified)"]}, {"type": "process_steps", "steps": [{"title": "Inspection", "description": "Site inspection for optimal placement", "step_number": 1}, {"title": "Installation", "description": "Mounting and wiring of the device", "step_number": 2}, {"title": "Configuration", "description": "Connecting the device to the smart network", "step_number": 3}, {"title": "Testing", "description": "Functional testing and system verification", "step_number": 4}, {"title": "Handover", "description": "Demonstrating usage and safety guidelines to the customer", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Do not touch exposed wiring before setup is complete", "Keep devices clean from dust"]}, {"type": "tools_materials", "tools": ["Drill machine", "Screwdrivers", "Wire strippers", "Mounting hardware"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure Wi-Fi availability", "Provide access to installation points"]}, {"type": "expected_results", "items": "Fully functional smart home system."}, {"type": "important_notes", "items": "Wi-Fi connectivity issues are not covered under installation warranty."}, {"type": "warranty", "details": "30 days service warranty.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "No, this is an installation service only unless specified.", "question": "Do you provide the devices?"}, {"answer": "Typically 1 to 2 hours depending on complexity.", "question": "How long does the installation take?"}, {"answer": "Yes, someone needs to be present to grant access and verify the setup.", "question": "Do I need to be home during the service?"}, {"answer": "Yes, we provide a 30-day service warranty on our work.", "question": "Is the installation covered by warranty?"}]}, {"type": "tips", "items": ["Change default passwords immediately after setup."]}, {"dos": ["Connect devices to a secure network."], "type": "dos_donts", "donts": ["Do not expose indoor cameras to outdoor environments."]}, {"type": "duration", "minutes": 60}]</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.827218+00:00</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.827218+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>498d667b-30bc-57fa-b3d2-7d7b1d46408f</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Video Doorbells Service Variation 1</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>6. Smart Home &amp; Security</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Video Doorbells</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>1200</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>["Standard installation", "Basic setup and testing", "Clean up post-service", "System demonstration"]</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>[{"text": "Professional video doorbells service for your smart home.", "type": "description"}, {"type": "highlights", "items": ["Expert Video Doorbells setup", "Secure configuration", "Post-installation demo", "24/7 Support available"]}, {"type": "excluded_scope", "items": ["Major structural modifications", "Cost of equipment (unless specified)"]}, {"type": "process_steps", "steps": [{"title": "Inspection", "description": "Site inspection for optimal placement", "step_number": 1}, {"title": "Installation", "description": "Mounting and wiring of the device", "step_number": 2}, {"title": "Configuration", "description": "Connecting the device to the smart network", "step_number": 3}, {"title": "Testing", "description": "Functional testing and system verification", "step_number": 4}, {"title": "Handover", "description": "Demonstrating usage and safety guidelines to the customer", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Do not touch exposed wiring before setup is complete", "Keep devices clean from dust"]}, {"type": "tools_materials", "tools": ["Drill machine", "Screwdrivers", "Wire strippers", "Mounting hardware"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure Wi-Fi availability", "Provide access to installation points"]}, {"type": "expected_results", "items": "Fully functional smart home system."}, {"type": "important_notes", "items": "Wi-Fi connectivity issues are not covered under installation warranty."}, {"type": "warranty", "details": "30 days service warranty.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "No, this is an installation service only unless specified.", "question": "Do you provide the devices?"}, {"answer": "Typically 1 to 2 hours depending on complexity.", "question": "How long does the installation take?"}, {"answer": "Yes, someone needs to be present to grant access and verify the setup.", "question": "Do I need to be home during the service?"}, {"answer": "Yes, we provide a 30-day service warranty on our work.", "question": "Is the installation covered by warranty?"}]}, {"type": "tips", "items": ["Change default passwords immediately after setup."]}, {"dos": ["Connect devices to a secure network."], "type": "dos_donts", "donts": ["Do not expose indoor cameras to outdoor environments."]}, {"type": "duration", "minutes": 60}]</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.830339+00:00</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.830339+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>f7b119f9-13b1-59f1-98e7-62a8a8d9273f</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Video Doorbells Service Variation 2</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>6. Smart Home &amp; Security</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Video Doorbells</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>1400</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>["Standard installation", "Basic setup and testing", "Clean up post-service", "System demonstration"]</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>[{"text": "Professional video doorbells service for your smart home.", "type": "description"}, {"type": "highlights", "items": ["Expert Video Doorbells setup", "Secure configuration", "Post-installation demo", "24/7 Support available"]}, {"type": "excluded_scope", "items": ["Major structural modifications", "Cost of equipment (unless specified)"]}, {"type": "process_steps", "steps": [{"title": "Inspection", "description": "Site inspection for optimal placement", "step_number": 1}, {"title": "Installation", "description": "Mounting and wiring of the device", "step_number": 2}, {"title": "Configuration", "description": "Connecting the device to the smart network", "step_number": 3}, {"title": "Testing", "description": "Functional testing and system verification", "step_number": 4}, {"title": "Handover", "description": "Demonstrating usage and safety guidelines to the customer", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Do not touch exposed wiring before setup is complete", "Keep devices clean from dust"]}, {"type": "tools_materials", "tools": ["Drill machine", "Screwdrivers", "Wire strippers", "Mounting hardware"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure Wi-Fi availability", "Provide access to installation points"]}, {"type": "expected_results", "items": "Fully functional smart home system."}, {"type": "important_notes", "items": "Wi-Fi connectivity issues are not covered under installation warranty."}, {"type": "warranty", "details": "30 days service warranty.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "No, this is an installation service only unless specified.", "question": "Do you provide the devices?"}, {"answer": "Typically 1 to 2 hours depending on complexity.", "question": "How long does the installation take?"}, {"answer": "Yes, someone needs to be present to grant access and verify the setup.", "question": "Do I need to be home during the service?"}, {"answer": "Yes, we provide a 30-day service warranty on our work.", "question": "Is the installation covered by warranty?"}]}, {"type": "tips", "items": ["Change default passwords immediately after setup."]}, {"dos": ["Connect devices to a secure network."], "type": "dos_donts", "donts": ["Do not expose indoor cameras to outdoor environments."]}, {"type": "duration", "minutes": 60}]</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.834067+00:00</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.834067+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>37cfa6a0-7a1d-52f2-9505-8c13fb818728</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Video Doorbells Service Variation 3</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>6. Smart Home &amp; Security</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Video Doorbells</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>1600</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>["Standard installation", "Basic setup and testing", "Clean up post-service", "System demonstration"]</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>[{"text": "Professional video doorbells service for your smart home.", "type": "description"}, {"type": "highlights", "items": ["Expert Video Doorbells setup", "Secure configuration", "Post-installation demo", "24/7 Support available"]}, {"type": "excluded_scope", "items": ["Major structural modifications", "Cost of equipment (unless specified)"]}, {"type": "process_steps", "steps": [{"title": "Inspection", "description": "Site inspection for optimal placement", "step_number": 1}, {"title": "Installation", "description": "Mounting and wiring of the device", "step_number": 2}, {"title": "Configuration", "description": "Connecting the device to the smart network", "step_number": 3}, {"title": "Testing", "description": "Functional testing and system verification", "step_number": 4}, {"title": "Handover", "description": "Demonstrating usage and safety guidelines to the customer", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Do not touch exposed wiring before setup is complete", "Keep devices clean from dust"]}, {"type": "tools_materials", "tools": ["Drill machine", "Screwdrivers", "Wire strippers", "Mounting hardware"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure Wi-Fi availability", "Provide access to installation points"]}, {"type": "expected_results", "items": "Fully functional smart home system."}, {"type": "important_notes", "items": "Wi-Fi connectivity issues are not covered under installation warranty."}, {"type": "warranty", "details": "30 days service warranty.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "No, this is an installation service only unless specified.", "question": "Do you provide the devices?"}, {"answer": "Typically 1 to 2 hours depending on complexity.", "question": "How long does the installation take?"}, {"answer": "Yes, someone needs to be present to grant access and verify the setup.", "question": "Do I need to be home during the service?"}, {"answer": "Yes, we provide a 30-day service warranty on our work.", "question": "Is the installation covered by warranty?"}]}, {"type": "tips", "items": ["Change default passwords immediately after setup."]}, {"dos": ["Connect devices to a secure network."], "type": "dos_donts", "donts": ["Do not expose indoor cameras to outdoor environments."]}, {"type": "duration", "minutes": 60}]</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.839062+00:00</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.839062+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>b24100aa-9570-547f-98cd-5d68c66dbddb</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Video Doorbells Service Variation 4</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>6. Smart Home &amp; Security</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Video Doorbells</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>1800</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>["Standard installation", "Basic setup and testing", "Clean up post-service", "System demonstration"]</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>[{"text": "Professional video doorbells service for your smart home.", "type": "description"}, {"type": "highlights", "items": ["Expert Video Doorbells setup", "Secure configuration", "Post-installation demo", "24/7 Support available"]}, {"type": "excluded_scope", "items": ["Major structural modifications", "Cost of equipment (unless specified)"]}, {"type": "process_steps", "steps": [{"title": "Inspection", "description": "Site inspection for optimal placement", "step_number": 1}, {"title": "Installation", "description": "Mounting and wiring of the device", "step_number": 2}, {"title": "Configuration", "description": "Connecting the device to the smart network", "step_number": 3}, {"title": "Testing", "description": "Functional testing and system verification", "step_number": 4}, {"title": "Handover", "description": "Demonstrating usage and safety guidelines to the customer", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Do not touch exposed wiring before setup is complete", "Keep devices clean from dust"]}, {"type": "tools_materials", "tools": ["Drill machine", "Screwdrivers", "Wire strippers", "Mounting hardware"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure Wi-Fi availability", "Provide access to installation points"]}, {"type": "expected_results", "items": "Fully functional smart home system."}, {"type": "important_notes", "items": "Wi-Fi connectivity issues are not covered under installation warranty."}, {"type": "warranty", "details": "30 days service warranty.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "No, this is an installation service only unless specified.", "question": "Do you provide the devices?"}, {"answer": "Typically 1 to 2 hours depending on complexity.", "question": "How long does the installation take?"}, {"answer": "Yes, someone needs to be present to grant access and verify the setup.", "question": "Do I need to be home during the service?"}, {"answer": "Yes, we provide a 30-day service warranty on our work.", "question": "Is the installation covered by warranty?"}]}, {"type": "tips", "items": ["Change default passwords immediately after setup."]}, {"dos": ["Connect devices to a secure network."], "type": "dos_donts", "donts": ["Do not expose indoor cameras to outdoor environments."]}, {"type": "duration", "minutes": 60}]</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.842148+00:00</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.842148+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>8e6d6f16-3511-5e08-bc92-35f12025e142</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Video Doorbells Service Variation 5</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>6. Smart Home &amp; Security</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Video Doorbells</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>["Standard installation", "Basic setup and testing", "Clean up post-service", "System demonstration"]</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>[{"text": "Professional video doorbells service for your smart home.", "type": "description"}, {"type": "highlights", "items": ["Expert Video Doorbells setup", "Secure configuration", "Post-installation demo", "24/7 Support available"]}, {"type": "excluded_scope", "items": ["Major structural modifications", "Cost of equipment (unless specified)"]}, {"type": "process_steps", "steps": [{"title": "Inspection", "description": "Site inspection for optimal placement", "step_number": 1}, {"title": "Installation", "description": "Mounting and wiring of the device", "step_number": 2}, {"title": "Configuration", "description": "Connecting the device to the smart network", "step_number": 3}, {"title": "Testing", "description": "Functional testing and system verification", "step_number": 4}, {"title": "Handover", "description": "Demonstrating usage and safety guidelines to the customer", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Do not touch exposed wiring before setup is complete", "Keep devices clean from dust"]}, {"type": "tools_materials", "tools": ["Drill machine", "Screwdrivers", "Wire strippers", "Mounting hardware"], "materials": []}, {"type": "customer_setup", "requirements": ["Ensure Wi-Fi availability", "Provide access to installation points"]}, {"type": "expected_results", "items": "Fully functional smart home system."}, {"type": "important_notes", "items": "Wi-Fi connectivity issues are not covered under installation warranty."}, {"type": "warranty", "details": "30 days service warranty.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "No, this is an installation service only unless specified.", "question": "Do you provide the devices?"}, {"answer": "Typically 1 to 2 hours depending on complexity.", "question": "How long does the installation take?"}, {"answer": "Yes, someone needs to be present to grant access and verify the setup.", "question": "Do I need to be home during the service?"}, {"answer": "Yes, we provide a 30-day service warranty on our work.", "question": "Is the installation covered by warranty?"}]}, {"type": "tips", "items": ["Change default passwords immediately after setup."]}, {"dos": ["Connect devices to a secure network."], "type": "dos_donts", "donts": ["Do not expose indoor cameras to outdoor environments."]}, {"type": "duration", "minutes": 60}]</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.845213+00:00</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>2026-09-05T14:33:06.845213+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>